<commit_message>
Improve dashboard analysis and demo data
</commit_message>
<xml_diff>
--- a/data/sample/paneer_quality_demo.xlsx
+++ b/data/sample/paneer_quality_demo.xlsx
@@ -417,45 +417,21 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr"/>
-      <c r="B1" t="inlineStr"/>
       <c r="C1" t="inlineStr">
         <is>
           <t>Synthetic demonstration data</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr"/>
-      <c r="E1" t="inlineStr"/>
-      <c r="F1" t="inlineStr"/>
-      <c r="G1" t="inlineStr"/>
       <c r="H1" t="inlineStr">
         <is>
           <t>Synthetic log10(CFU/mL)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr"/>
-      <c r="J1" t="inlineStr"/>
-      <c r="K1" t="inlineStr"/>
-      <c r="L1" t="inlineStr"/>
-      <c r="M1" t="inlineStr"/>
-      <c r="N1" t="inlineStr"/>
-      <c r="O1" t="inlineStr"/>
       <c r="P1" t="inlineStr">
         <is>
           <t>Synthetic sensory scores</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr"/>
-      <c r="R1" t="inlineStr"/>
-      <c r="S1" t="inlineStr"/>
-      <c r="T1" t="inlineStr"/>
-      <c r="U1" t="inlineStr"/>
-      <c r="V1" t="inlineStr"/>
-      <c r="W1" t="inlineStr"/>
-      <c r="X1" t="inlineStr"/>
-      <c r="Y1" t="inlineStr"/>
-      <c r="Z1" t="inlineStr"/>
-      <c r="AA1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -528,7 +504,6 @@
           <t>Psychrophilic count</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr"/>
       <c r="P2" t="inlineStr">
         <is>
           <t>Colour and Appearance</t>
@@ -549,7 +524,6 @@
           <t>Overall Acceptability</t>
         </is>
       </c>
-      <c r="T2" t="inlineStr"/>
       <c r="U2" t="inlineStr">
         <is>
           <t>pH</t>
@@ -560,7 +534,6 @@
           <t>Moisture %</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr"/>
       <c r="X2" t="inlineStr">
         <is>
           <t>Milk</t>
@@ -596,7 +569,7 @@
         <v>1</v>
       </c>
       <c r="E3" t="n">
-        <v>2.210050849875137</v>
+        <v>2.517</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
@@ -604,22 +577,18 @@
       <c r="G3" t="n">
         <v>1</v>
       </c>
-      <c r="H3" t="inlineStr"/>
       <c r="I3" t="n">
         <v>0</v>
       </c>
       <c r="J3" t="n">
         <v>1</v>
       </c>
-      <c r="K3" t="inlineStr"/>
       <c r="L3" t="n">
         <v>0</v>
       </c>
       <c r="M3" t="n">
         <v>1</v>
       </c>
-      <c r="N3" t="inlineStr"/>
-      <c r="O3" t="inlineStr"/>
       <c r="P3" t="n">
         <v>8.720000000000001</v>
       </c>
@@ -630,16 +599,14 @@
         <v>8.67</v>
       </c>
       <c r="S3" t="n">
-        <v>8.637</v>
-      </c>
-      <c r="T3" t="inlineStr"/>
+        <v>8.957000000000001</v>
+      </c>
       <c r="U3" t="n">
         <v>5.68</v>
       </c>
       <c r="V3" t="n">
         <v>53.06</v>
       </c>
-      <c r="W3" t="inlineStr"/>
       <c r="X3" t="n">
         <v>10.1</v>
       </c>
@@ -667,7 +634,7 @@
         <v>1</v>
       </c>
       <c r="E4" t="n">
-        <v>2.279894980011638</v>
+        <v>2.312</v>
       </c>
       <c r="F4" t="n">
         <v>0.24</v>
@@ -696,7 +663,6 @@
       <c r="N4" t="n">
         <v>0.5314789170422551</v>
       </c>
-      <c r="O4" t="inlineStr"/>
       <c r="P4" t="n">
         <v>8.859999999999999</v>
       </c>
@@ -707,16 +673,14 @@
         <v>8.81</v>
       </c>
       <c r="S4" t="n">
-        <v>8.776999999999999</v>
-      </c>
-      <c r="T4" t="inlineStr"/>
+        <v>9.026</v>
+      </c>
       <c r="U4" t="n">
         <v>5.7</v>
       </c>
       <c r="V4" t="n">
         <v>53.13</v>
       </c>
-      <c r="W4" t="inlineStr"/>
       <c r="X4" t="n">
         <v>10.2</v>
       </c>
@@ -744,7 +708,7 @@
         <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>2.35005409357903</v>
+        <v>2.252</v>
       </c>
       <c r="F5" t="n">
         <v>0.28</v>
@@ -773,7 +737,6 @@
       <c r="N5" t="n">
         <v>0.6020599913279624</v>
       </c>
-      <c r="O5" t="inlineStr"/>
       <c r="P5" t="n">
         <v>9</v>
       </c>
@@ -784,16 +747,14 @@
         <v>8.949999999999999</v>
       </c>
       <c r="S5" t="n">
-        <v>8.917</v>
-      </c>
-      <c r="T5" t="inlineStr"/>
+        <v>8.552</v>
+      </c>
       <c r="U5" t="n">
         <v>5.72</v>
       </c>
       <c r="V5" t="n">
         <v>53.2</v>
       </c>
-      <c r="W5" t="inlineStr"/>
       <c r="X5" t="n">
         <v>10.3</v>
       </c>
@@ -821,7 +782,7 @@
         <v>1</v>
       </c>
       <c r="E6" t="n">
-        <v>2.419955748489758</v>
+        <v>2.259</v>
       </c>
       <c r="F6" t="n">
         <v>0.33</v>
@@ -850,7 +811,6 @@
       <c r="N6" t="n">
         <v>0.6720978579357174</v>
       </c>
-      <c r="O6" t="inlineStr"/>
       <c r="P6" t="n">
         <v>9.140000000000001</v>
       </c>
@@ -861,16 +821,14 @@
         <v>9.09</v>
       </c>
       <c r="S6" t="n">
-        <v>9.057</v>
-      </c>
-      <c r="T6" t="inlineStr"/>
+        <v>9.327999999999999</v>
+      </c>
       <c r="U6" t="n">
         <v>5.74</v>
       </c>
       <c r="V6" t="n">
         <v>53.27</v>
       </c>
-      <c r="W6" t="inlineStr"/>
       <c r="X6" t="n">
         <v>10.4</v>
       </c>
@@ -898,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="E7" t="n">
-        <v>2.489958479424835</v>
+        <v>2.376</v>
       </c>
       <c r="F7" t="n">
         <v>0.39</v>
@@ -927,7 +885,6 @@
       <c r="N7" t="n">
         <v>0.7403626894942439</v>
       </c>
-      <c r="O7" t="inlineStr"/>
       <c r="P7" t="n">
         <v>9.279999999999999</v>
       </c>
@@ -938,16 +895,14 @@
         <v>9.23</v>
       </c>
       <c r="S7" t="n">
-        <v>9.196999999999999</v>
-      </c>
-      <c r="T7" t="inlineStr"/>
+        <v>8.555999999999999</v>
+      </c>
       <c r="U7" t="n">
         <v>5.75</v>
       </c>
       <c r="V7" t="n">
         <v>53.34</v>
       </c>
-      <c r="W7" t="inlineStr"/>
       <c r="X7" t="n">
         <v>10.5</v>
       </c>
@@ -975,7 +930,7 @@
         <v>1</v>
       </c>
       <c r="E8" t="n">
-        <v>2.510008512940235</v>
+        <v>2.632</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
@@ -983,22 +938,18 @@
       <c r="G8" t="n">
         <v>1</v>
       </c>
-      <c r="H8" t="inlineStr"/>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
         <v>1</v>
       </c>
-      <c r="K8" t="inlineStr"/>
       <c r="L8" t="n">
         <v>0</v>
       </c>
       <c r="M8" t="n">
         <v>1</v>
       </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
       <c r="P8" t="n">
         <v>8.289999999999999</v>
       </c>
@@ -1009,20 +960,14 @@
         <v>8.24</v>
       </c>
       <c r="S8" t="n">
-        <v>8.207000000000001</v>
-      </c>
-      <c r="T8" t="inlineStr"/>
+        <v>8.775</v>
+      </c>
       <c r="U8" t="n">
         <v>5.71</v>
       </c>
       <c r="V8" t="n">
         <v>52.9</v>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
-      <c r="Y8" t="inlineStr"/>
-      <c r="Z8" t="inlineStr"/>
-      <c r="AA8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -1038,7 +983,7 @@
         <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>2.580012112529424</v>
+        <v>2.615</v>
       </c>
       <c r="F9" t="n">
         <v>0.37</v>
@@ -1067,7 +1012,6 @@
       <c r="N9" t="n">
         <v>0.7075701760979364</v>
       </c>
-      <c r="O9" t="inlineStr"/>
       <c r="P9" t="n">
         <v>8.43</v>
       </c>
@@ -1078,20 +1022,14 @@
         <v>8.380000000000001</v>
       </c>
       <c r="S9" t="n">
-        <v>8.347</v>
-      </c>
-      <c r="T9" t="inlineStr"/>
+        <v>8.125999999999999</v>
+      </c>
       <c r="U9" t="n">
         <v>5.73</v>
       </c>
       <c r="V9" t="n">
         <v>52.97</v>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
-      <c r="Y9" t="inlineStr"/>
-      <c r="Z9" t="inlineStr"/>
-      <c r="AA9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -1107,7 +1045,7 @@
         <v>1</v>
       </c>
       <c r="E10" t="n">
-        <v>2.650015952471839</v>
+        <v>2.692</v>
       </c>
       <c r="F10" t="n">
         <v>0.44</v>
@@ -1136,7 +1074,6 @@
       <c r="N10" t="n">
         <v>0.7781512503836435</v>
       </c>
-      <c r="O10" t="inlineStr"/>
       <c r="P10" t="n">
         <v>8.57</v>
       </c>
@@ -1147,20 +1084,14 @@
         <v>8.52</v>
       </c>
       <c r="S10" t="n">
-        <v>8.487</v>
-      </c>
-      <c r="T10" t="inlineStr"/>
+        <v>8.196</v>
+      </c>
       <c r="U10" t="n">
         <v>5.75</v>
       </c>
       <c r="V10" t="n">
         <v>53.04</v>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
-      <c r="Y10" t="inlineStr"/>
-      <c r="Z10" t="inlineStr"/>
-      <c r="AA10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -1176,7 +1107,7 @@
         <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>2.719993826367604</v>
+        <v>2.699</v>
       </c>
       <c r="F11" t="n">
         <v>0.51</v>
@@ -1205,7 +1136,6 @@
       <c r="N11" t="n">
         <v>0.8512583487190752</v>
       </c>
-      <c r="O11" t="inlineStr"/>
       <c r="P11" t="n">
         <v>8.710000000000001</v>
       </c>
@@ -1216,20 +1146,14 @@
         <v>8.66</v>
       </c>
       <c r="S11" t="n">
-        <v>8.627000000000001</v>
-      </c>
-      <c r="T11" t="inlineStr"/>
+        <v>8.315</v>
+      </c>
       <c r="U11" t="n">
         <v>5.76</v>
       </c>
       <c r="V11" t="n">
         <v>53.11</v>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
-      <c r="Y11" t="inlineStr"/>
-      <c r="Z11" t="inlineStr"/>
-      <c r="AA11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -1245,7 +1169,7 @@
         <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>2.790003520390489</v>
+        <v>2.582</v>
       </c>
       <c r="F12" t="n">
         <v>0.6</v>
@@ -1274,7 +1198,6 @@
       <c r="N12" t="n">
         <v>0.9190780923760739</v>
       </c>
-      <c r="O12" t="inlineStr"/>
       <c r="P12" t="n">
         <v>8.85</v>
       </c>
@@ -1285,20 +1208,14 @@
         <v>8.800000000000001</v>
       </c>
       <c r="S12" t="n">
-        <v>8.766999999999999</v>
-      </c>
-      <c r="T12" t="inlineStr"/>
+        <v>8.750999999999999</v>
+      </c>
       <c r="U12" t="n">
         <v>5.78</v>
       </c>
       <c r="V12" t="n">
         <v>53.18</v>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
-      <c r="Y12" t="inlineStr"/>
-      <c r="Z12" t="inlineStr"/>
-      <c r="AA12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -1314,7 +1231,7 @@
         <v>1</v>
       </c>
       <c r="E13" t="n">
-        <v>2.810030786405839</v>
+        <v>2.908</v>
       </c>
       <c r="F13" t="n">
         <v>0.49</v>
@@ -1343,7 +1260,6 @@
       <c r="N13" t="n">
         <v>0.8195439355418687</v>
       </c>
-      <c r="O13" t="inlineStr"/>
       <c r="P13" t="n">
         <v>7.86</v>
       </c>
@@ -1354,20 +1270,14 @@
         <v>7.81</v>
       </c>
       <c r="S13" t="n">
-        <v>7.777</v>
-      </c>
-      <c r="T13" t="inlineStr"/>
+        <v>7.115</v>
+      </c>
       <c r="U13" t="n">
         <v>5.73</v>
       </c>
       <c r="V13" t="n">
         <v>52.74</v>
       </c>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
-      <c r="Y13" t="inlineStr"/>
-      <c r="Z13" t="inlineStr"/>
-      <c r="AA13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -1383,7 +1293,7 @@
         <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>2.880012838366772</v>
+        <v>3.077</v>
       </c>
       <c r="F14" t="n">
         <v>0.58</v>
@@ -1412,7 +1322,6 @@
       <c r="N14" t="n">
         <v>0.8920946026904804</v>
       </c>
-      <c r="O14" t="inlineStr"/>
       <c r="P14" t="n">
         <v>8</v>
       </c>
@@ -1423,20 +1332,14 @@
         <v>7.95</v>
       </c>
       <c r="S14" t="n">
-        <v>7.917</v>
-      </c>
-      <c r="T14" t="inlineStr"/>
+        <v>8.388</v>
+      </c>
       <c r="U14" t="n">
         <v>5.75</v>
       </c>
       <c r="V14" t="n">
         <v>52.81</v>
       </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
-      <c r="Y14" t="inlineStr"/>
-      <c r="Z14" t="inlineStr"/>
-      <c r="AA14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -1452,7 +1355,7 @@
         <v>1</v>
       </c>
       <c r="E15" t="n">
-        <v>2.950023906523326</v>
+        <v>2.947</v>
       </c>
       <c r="F15" t="n">
         <v>0.68</v>
@@ -1481,7 +1384,6 @@
       <c r="N15" t="n">
         <v>0.9590413923210935</v>
       </c>
-      <c r="O15" t="inlineStr"/>
       <c r="P15" t="n">
         <v>8.140000000000001</v>
       </c>
@@ -1492,20 +1394,14 @@
         <v>8.09</v>
       </c>
       <c r="S15" t="n">
-        <v>8.057</v>
-      </c>
-      <c r="T15" t="inlineStr"/>
+        <v>8.537000000000001</v>
+      </c>
       <c r="U15" t="n">
         <v>5.77</v>
       </c>
       <c r="V15" t="n">
         <v>52.88</v>
       </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
-      <c r="Y15" t="inlineStr"/>
-      <c r="Z15" t="inlineStr"/>
-      <c r="AA15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -1521,7 +1417,7 @@
         <v>1</v>
       </c>
       <c r="E16" t="n">
-        <v>3.019988159591285</v>
+        <v>2.93</v>
       </c>
       <c r="F16" t="n">
         <v>0.79</v>
@@ -1550,7 +1446,6 @@
       <c r="N16" t="n">
         <v>1.02938377768521</v>
       </c>
-      <c r="O16" t="inlineStr"/>
       <c r="P16" t="n">
         <v>8.279999999999999</v>
       </c>
@@ -1561,20 +1456,14 @@
         <v>8.23</v>
       </c>
       <c r="S16" t="n">
-        <v>8.196999999999999</v>
-      </c>
-      <c r="T16" t="inlineStr"/>
+        <v>8.205</v>
+      </c>
       <c r="U16" t="n">
         <v>5.79</v>
       </c>
       <c r="V16" t="n">
         <v>52.95</v>
       </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
-      <c r="Y16" t="inlineStr"/>
-      <c r="Z16" t="inlineStr"/>
-      <c r="AA16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -1590,7 +1479,7 @@
         <v>1</v>
       </c>
       <c r="E17" t="n">
-        <v>3.090011024007147</v>
+        <v>2.984</v>
       </c>
       <c r="F17" t="n">
         <v>0.93</v>
@@ -1619,7 +1508,6 @@
       <c r="N17" t="n">
         <v>1.100370545117563</v>
       </c>
-      <c r="O17" t="inlineStr"/>
       <c r="P17" t="n">
         <v>8.42</v>
       </c>
@@ -1630,20 +1518,14 @@
         <v>8.369999999999999</v>
       </c>
       <c r="S17" t="n">
-        <v>8.337</v>
-      </c>
-      <c r="T17" t="inlineStr"/>
+        <v>7.804</v>
+      </c>
       <c r="U17" t="n">
         <v>5.8</v>
       </c>
       <c r="V17" t="n">
         <v>53.02</v>
       </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
-      <c r="Y17" t="inlineStr"/>
-      <c r="Z17" t="inlineStr"/>
-      <c r="AA17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -1659,7 +1541,7 @@
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>3.109983294819892</v>
+        <v>3.197</v>
       </c>
       <c r="F18" t="n">
         <v>0.76</v>
@@ -1688,7 +1570,6 @@
       <c r="N18" t="n">
         <v>1</v>
       </c>
-      <c r="O18" t="inlineStr"/>
       <c r="P18" t="n">
         <v>7.43</v>
       </c>
@@ -1699,20 +1580,14 @@
         <v>7.38</v>
       </c>
       <c r="S18" t="n">
-        <v>7.347</v>
-      </c>
-      <c r="T18" t="inlineStr"/>
+        <v>6.892</v>
+      </c>
       <c r="U18" t="n">
         <v>5.76</v>
       </c>
       <c r="V18" t="n">
         <v>52.58</v>
       </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
-      <c r="Y18" t="inlineStr"/>
-      <c r="Z18" t="inlineStr"/>
-      <c r="AA18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -1728,7 +1603,7 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>3.180011119057717</v>
+        <v>3.189</v>
       </c>
       <c r="F19" t="n">
         <v>0.89</v>
@@ -1757,7 +1632,6 @@
       <c r="N19" t="n">
         <v>1.068185861746162</v>
       </c>
-      <c r="O19" t="inlineStr"/>
       <c r="P19" t="n">
         <v>7.57</v>
       </c>
@@ -1768,20 +1642,14 @@
         <v>7.52</v>
       </c>
       <c r="S19" t="n">
-        <v>7.487</v>
-      </c>
-      <c r="T19" t="inlineStr"/>
+        <v>7.128</v>
+      </c>
       <c r="U19" t="n">
         <v>5.78</v>
       </c>
       <c r="V19" t="n">
         <v>52.65</v>
       </c>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
-      <c r="Y19" t="inlineStr"/>
-      <c r="Z19" t="inlineStr"/>
-      <c r="AA19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -1797,7 +1665,7 @@
         <v>1</v>
       </c>
       <c r="E20" t="n">
-        <v>3.250005028486896</v>
+        <v>3.186</v>
       </c>
       <c r="F20" t="n">
         <v>1.05</v>
@@ -1826,7 +1694,6 @@
       <c r="N20" t="n">
         <v>1.139879086401236</v>
       </c>
-      <c r="O20" t="inlineStr"/>
       <c r="P20" t="n">
         <v>7.71</v>
       </c>
@@ -1837,20 +1704,14 @@
         <v>7.66</v>
       </c>
       <c r="S20" t="n">
-        <v>7.627</v>
-      </c>
-      <c r="T20" t="inlineStr"/>
+        <v>7.331</v>
+      </c>
       <c r="U20" t="n">
         <v>5.79</v>
       </c>
       <c r="V20" t="n">
         <v>52.72</v>
       </c>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
-      <c r="Y20" t="inlineStr"/>
-      <c r="Z20" t="inlineStr"/>
-      <c r="AA20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -1866,7 +1727,7 @@
         <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>3.320000804264728</v>
+        <v>3.347</v>
       </c>
       <c r="F21" t="n">
         <v>1.23</v>
@@ -1895,7 +1756,6 @@
       <c r="N21" t="n">
         <v>1.209515014542631</v>
       </c>
-      <c r="O21" t="inlineStr"/>
       <c r="P21" t="n">
         <v>7.85</v>
       </c>
@@ -1906,20 +1766,14 @@
         <v>7.8</v>
       </c>
       <c r="S21" t="n">
-        <v>7.767</v>
-      </c>
-      <c r="T21" t="inlineStr"/>
+        <v>8.308</v>
+      </c>
       <c r="U21" t="n">
         <v>5.81</v>
       </c>
       <c r="V21" t="n">
         <v>52.79</v>
       </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
-      <c r="Y21" t="inlineStr"/>
-      <c r="Z21" t="inlineStr"/>
-      <c r="AA21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1935,7 +1789,7 @@
         <v>1</v>
       </c>
       <c r="E22" t="n">
-        <v>3.389998422607333</v>
+        <v>3.272</v>
       </c>
       <c r="F22" t="n">
         <v>1.45</v>
@@ -1964,7 +1818,6 @@
       <c r="N22" t="n">
         <v>1.281033367247727</v>
       </c>
-      <c r="O22" t="inlineStr"/>
       <c r="P22" t="n">
         <v>7.99</v>
       </c>
@@ -1975,20 +1828,14 @@
         <v>7.94</v>
       </c>
       <c r="S22" t="n">
-        <v>7.907</v>
-      </c>
-      <c r="T22" t="inlineStr"/>
+        <v>7.318</v>
+      </c>
       <c r="U22" t="n">
         <v>5.83</v>
       </c>
       <c r="V22" t="n">
         <v>52.86</v>
       </c>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
-      <c r="Y22" t="inlineStr"/>
-      <c r="Z22" t="inlineStr"/>
-      <c r="AA22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -2004,7 +1851,7 @@
         <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>3.410000712543462</v>
+        <v>3.492</v>
       </c>
       <c r="F23" t="n">
         <v>1.17</v>
@@ -2033,7 +1880,6 @@
       <c r="N23" t="n">
         <v>1.178976947293169</v>
       </c>
-      <c r="O23" t="inlineStr"/>
       <c r="P23" t="n">
         <v>7</v>
       </c>
@@ -2044,20 +1890,14 @@
         <v>6.95</v>
       </c>
       <c r="S23" t="n">
-        <v>6.917</v>
-      </c>
-      <c r="T23" t="inlineStr"/>
+        <v>7.225</v>
+      </c>
       <c r="U23" t="n">
         <v>5.78</v>
       </c>
       <c r="V23" t="n">
         <v>52.42</v>
       </c>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
-      <c r="Y23" t="inlineStr"/>
-      <c r="Z23" t="inlineStr"/>
-      <c r="AA23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -2073,7 +1913,7 @@
         <v>1</v>
       </c>
       <c r="E24" t="n">
-        <v>3.480006942957151</v>
+        <v>3.677</v>
       </c>
       <c r="F24" t="n">
         <v>1.38</v>
@@ -2102,7 +1942,6 @@
       <c r="N24" t="n">
         <v>1.250420002308894</v>
       </c>
-      <c r="O24" t="inlineStr"/>
       <c r="P24" t="n">
         <v>7.14</v>
       </c>
@@ -2113,20 +1952,14 @@
         <v>7.09</v>
       </c>
       <c r="S24" t="n">
-        <v>7.057</v>
-      </c>
-      <c r="T24" t="inlineStr"/>
+        <v>7.5</v>
+      </c>
       <c r="U24" t="n">
         <v>5.8</v>
       </c>
       <c r="V24" t="n">
         <v>52.49</v>
       </c>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
-      <c r="Y24" t="inlineStr"/>
-      <c r="Z24" t="inlineStr"/>
-      <c r="AA24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -2142,7 +1975,7 @@
         <v>1</v>
       </c>
       <c r="E25" t="n">
-        <v>3.549995851530651</v>
+        <v>3.478</v>
       </c>
       <c r="F25" t="n">
         <v>1.62</v>
@@ -2171,7 +2004,6 @@
       <c r="N25" t="n">
         <v>1.320146286111054</v>
       </c>
-      <c r="O25" t="inlineStr"/>
       <c r="P25" t="n">
         <v>7.28</v>
       </c>
@@ -2182,20 +2014,14 @@
         <v>7.23</v>
       </c>
       <c r="S25" t="n">
-        <v>7.197</v>
-      </c>
-      <c r="T25" t="inlineStr"/>
+        <v>7.493</v>
+      </c>
       <c r="U25" t="n">
         <v>5.82</v>
       </c>
       <c r="V25" t="n">
         <v>52.56</v>
       </c>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
-      <c r="Y25" t="inlineStr"/>
-      <c r="Z25" t="inlineStr"/>
-      <c r="AA25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -2211,7 +2037,7 @@
         <v>1</v>
       </c>
       <c r="E26" t="n">
-        <v>3.620000642300068</v>
+        <v>3.476</v>
       </c>
       <c r="F26" t="n">
         <v>1.91</v>
@@ -2240,7 +2066,6 @@
       <c r="N26" t="n">
         <v>1.389166084364532</v>
       </c>
-      <c r="O26" t="inlineStr"/>
       <c r="P26" t="n">
         <v>7.42</v>
       </c>
@@ -2251,20 +2076,14 @@
         <v>7.37</v>
       </c>
       <c r="S26" t="n">
-        <v>7.337</v>
-      </c>
-      <c r="T26" t="inlineStr"/>
+        <v>6.852</v>
+      </c>
       <c r="U26" t="n">
         <v>5.84</v>
       </c>
       <c r="V26" t="n">
         <v>52.63</v>
       </c>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
-      <c r="Y26" t="inlineStr"/>
-      <c r="Z26" t="inlineStr"/>
-      <c r="AA26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -2280,7 +2099,7 @@
         <v>1</v>
       </c>
       <c r="E27" t="n">
-        <v>3.690001046883064</v>
+        <v>3.61</v>
       </c>
       <c r="F27" t="n">
         <v>0</v>
@@ -2288,22 +2107,18 @@
       <c r="G27" t="n">
         <v>1</v>
       </c>
-      <c r="H27" t="inlineStr"/>
       <c r="I27" t="n">
         <v>0</v>
       </c>
       <c r="J27" t="n">
         <v>1</v>
       </c>
-      <c r="K27" t="inlineStr"/>
       <c r="L27" t="n">
         <v>0</v>
       </c>
       <c r="M27" t="n">
         <v>1</v>
       </c>
-      <c r="N27" t="inlineStr"/>
-      <c r="O27" t="inlineStr"/>
       <c r="P27" t="n">
         <v>7.56</v>
       </c>
@@ -2314,20 +2129,14 @@
         <v>7.51</v>
       </c>
       <c r="S27" t="n">
-        <v>7.477</v>
-      </c>
-      <c r="T27" t="inlineStr"/>
+        <v>7.279</v>
+      </c>
       <c r="U27" t="n">
         <v>5.85</v>
       </c>
       <c r="V27" t="n">
         <v>52.7</v>
       </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
-      <c r="Y27" t="inlineStr"/>
-      <c r="Z27" t="inlineStr"/>
-      <c r="AA27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -2343,7 +2152,7 @@
         <v>1</v>
       </c>
       <c r="E28" t="n">
-        <v>3.709998828025189</v>
+        <v>3.738</v>
       </c>
       <c r="F28" t="n">
         <v>1.82</v>
@@ -2372,7 +2181,6 @@
       <c r="N28" t="n">
         <v>1.359835482339888</v>
       </c>
-      <c r="O28" t="inlineStr"/>
       <c r="P28" t="n">
         <v>6.57</v>
       </c>
@@ -2383,20 +2191,14 @@
         <v>6.52</v>
       </c>
       <c r="S28" t="n">
-        <v>6.487</v>
-      </c>
-      <c r="T28" t="inlineStr"/>
+        <v>6.72</v>
+      </c>
       <c r="U28" t="n">
         <v>5.81</v>
       </c>
       <c r="V28" t="n">
         <v>52.26</v>
       </c>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
-      <c r="Y28" t="inlineStr"/>
-      <c r="Z28" t="inlineStr"/>
-      <c r="AA28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -2412,7 +2214,7 @@
         <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>3.780000298336571</v>
+        <v>3.934</v>
       </c>
       <c r="F29" t="n">
         <v>2.14</v>
@@ -2441,7 +2243,6 @@
       <c r="N29" t="n">
         <v>1.429752280002408</v>
       </c>
-      <c r="O29" t="inlineStr"/>
       <c r="P29" t="n">
         <v>6.71</v>
       </c>
@@ -2452,20 +2253,14 @@
         <v>6.66</v>
       </c>
       <c r="S29" t="n">
-        <v>6.627</v>
-      </c>
-      <c r="T29" t="inlineStr"/>
+        <v>6.241</v>
+      </c>
       <c r="U29" t="n">
         <v>5.83</v>
       </c>
       <c r="V29" t="n">
         <v>52.33</v>
       </c>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
-      <c r="Y29" t="inlineStr"/>
-      <c r="Z29" t="inlineStr"/>
-      <c r="AA29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -2481,7 +2276,7 @@
         <v>1</v>
       </c>
       <c r="E30" t="n">
-        <v>3.850002586092461</v>
+        <v>3.754</v>
       </c>
       <c r="F30" t="n">
         <v>2.51</v>
@@ -2510,7 +2305,6 @@
       <c r="N30" t="n">
         <v>1.499687082618404</v>
       </c>
-      <c r="O30" t="inlineStr"/>
       <c r="P30" t="n">
         <v>6.85</v>
       </c>
@@ -2521,20 +2315,14 @@
         <v>6.8</v>
       </c>
       <c r="S30" t="n">
-        <v>6.767</v>
-      </c>
-      <c r="T30" t="inlineStr"/>
+        <v>6.896</v>
+      </c>
       <c r="U30" t="n">
         <v>5.84</v>
       </c>
       <c r="V30" t="n">
         <v>52.4</v>
       </c>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
-      <c r="Y30" t="inlineStr"/>
-      <c r="Z30" t="inlineStr"/>
-      <c r="AA30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -2550,7 +2338,7 @@
         <v>1</v>
       </c>
       <c r="E31" t="n">
-        <v>3.919998030964019</v>
+        <v>3.825</v>
       </c>
       <c r="F31" t="n">
         <v>0</v>
@@ -2558,22 +2346,18 @@
       <c r="G31" t="n">
         <v>1</v>
       </c>
-      <c r="H31" t="inlineStr"/>
       <c r="I31" t="n">
         <v>0</v>
       </c>
       <c r="J31" t="n">
         <v>1</v>
       </c>
-      <c r="K31" t="inlineStr"/>
       <c r="L31" t="n">
         <v>0</v>
       </c>
       <c r="M31" t="n">
         <v>1</v>
       </c>
-      <c r="N31" t="inlineStr"/>
-      <c r="O31" t="inlineStr"/>
       <c r="P31" t="n">
         <v>6.99</v>
       </c>
@@ -2584,20 +2368,14 @@
         <v>6.94</v>
       </c>
       <c r="S31" t="n">
-        <v>6.907</v>
-      </c>
-      <c r="T31" t="inlineStr"/>
+        <v>6.651</v>
+      </c>
       <c r="U31" t="n">
         <v>5.86</v>
       </c>
       <c r="V31" t="n">
         <v>52.47</v>
       </c>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
-      <c r="Y31" t="inlineStr"/>
-      <c r="Z31" t="inlineStr"/>
-      <c r="AA31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -2613,7 +2391,7 @@
         <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>3.990001235034661</v>
+        <v>3.813</v>
       </c>
       <c r="F32" t="n">
         <v>3.47</v>
@@ -2642,7 +2420,6 @@
       <c r="N32" t="n">
         <v>1.640481436970422</v>
       </c>
-      <c r="O32" t="inlineStr"/>
       <c r="P32" t="n">
         <v>7.13</v>
       </c>
@@ -2653,20 +2430,14 @@
         <v>7.08</v>
       </c>
       <c r="S32" t="n">
-        <v>7.047</v>
-      </c>
-      <c r="T32" t="inlineStr"/>
+        <v>6.742</v>
+      </c>
       <c r="U32" t="n">
         <v>5.88</v>
       </c>
       <c r="V32" t="n">
         <v>52.54</v>
       </c>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
-      <c r="Y32" t="inlineStr"/>
-      <c r="Z32" t="inlineStr"/>
-      <c r="AA32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -2682,7 +2453,7 @@
         <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>4.009998730048061</v>
+        <v>4.052</v>
       </c>
       <c r="F33" t="n">
         <v>2.82</v>
@@ -2711,7 +2482,6 @@
       <c r="N33" t="n">
         <v>1.540329474790874</v>
       </c>
-      <c r="O33" t="inlineStr"/>
       <c r="P33" t="n">
         <v>6.14</v>
       </c>
@@ -2722,20 +2492,14 @@
         <v>6.09</v>
       </c>
       <c r="S33" t="n">
-        <v>6.057</v>
-      </c>
-      <c r="T33" t="inlineStr"/>
+        <v>6.121</v>
+      </c>
       <c r="U33" t="n">
         <v>5.83</v>
       </c>
       <c r="V33" t="n">
         <v>52.1</v>
       </c>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
-      <c r="Y33" t="inlineStr"/>
-      <c r="Z33" t="inlineStr"/>
-      <c r="AA33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -2751,7 +2515,7 @@
         <v>1</v>
       </c>
       <c r="E34" t="n">
-        <v>4.079998398078352</v>
+        <v>4.263</v>
       </c>
       <c r="F34" t="n">
         <v>3.31</v>
@@ -2780,7 +2544,6 @@
       <c r="N34" t="n">
         <v>1.60959440922522</v>
       </c>
-      <c r="O34" t="inlineStr"/>
       <c r="P34" t="n">
         <v>6.28</v>
       </c>
@@ -2791,20 +2554,14 @@
         <v>6.23</v>
       </c>
       <c r="S34" t="n">
-        <v>6.197</v>
-      </c>
-      <c r="T34" t="inlineStr"/>
+        <v>6.235</v>
+      </c>
       <c r="U34" t="n">
         <v>5.85</v>
       </c>
       <c r="V34" t="n">
         <v>52.17</v>
       </c>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
-      <c r="Y34" t="inlineStr"/>
-      <c r="Z34" t="inlineStr"/>
-      <c r="AA34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -2820,7 +2577,7 @@
         <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>4.150000754922137</v>
+        <v>4.175</v>
       </c>
       <c r="F35" t="n">
         <v>0</v>
@@ -2828,22 +2585,18 @@
       <c r="G35" t="n">
         <v>1</v>
       </c>
-      <c r="H35" t="inlineStr"/>
       <c r="I35" t="n">
         <v>0</v>
       </c>
       <c r="J35" t="n">
         <v>1</v>
       </c>
-      <c r="K35" t="inlineStr"/>
       <c r="L35" t="n">
         <v>0</v>
       </c>
       <c r="M35" t="n">
         <v>1</v>
       </c>
-      <c r="N35" t="inlineStr"/>
-      <c r="O35" t="inlineStr"/>
       <c r="P35" t="n">
         <v>6.42</v>
       </c>
@@ -2854,20 +2607,14 @@
         <v>6.37</v>
       </c>
       <c r="S35" t="n">
-        <v>6.337</v>
-      </c>
-      <c r="T35" t="inlineStr"/>
+        <v>6.189</v>
+      </c>
       <c r="U35" t="n">
         <v>5.87</v>
       </c>
       <c r="V35" t="n">
         <v>52.24</v>
       </c>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
-      <c r="Y35" t="inlineStr"/>
-      <c r="Z35" t="inlineStr"/>
-      <c r="AA35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -2883,7 +2630,7 @@
         <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>4.220000809286663</v>
+        <v>4.022</v>
       </c>
       <c r="F36" t="n">
         <v>4.57</v>
@@ -2912,7 +2659,6 @@
       <c r="N36" t="n">
         <v>1.749736315569061</v>
       </c>
-      <c r="O36" t="inlineStr"/>
       <c r="P36" t="n">
         <v>6.56</v>
       </c>
@@ -2923,20 +2669,14 @@
         <v>6.51</v>
       </c>
       <c r="S36" t="n">
-        <v>6.477</v>
-      </c>
-      <c r="T36" t="inlineStr"/>
+        <v>6.272</v>
+      </c>
       <c r="U36" t="n">
         <v>5.89</v>
       </c>
       <c r="V36" t="n">
         <v>52.31</v>
       </c>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
-      <c r="Y36" t="inlineStr"/>
-      <c r="Z36" t="inlineStr"/>
-      <c r="AA36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -2952,7 +2692,7 @@
         <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>4.289998975481486</v>
+        <v>4.142</v>
       </c>
       <c r="F37" t="n">
         <v>5.37</v>
@@ -2981,7 +2721,6 @@
       <c r="N37" t="n">
         <v>1.82020145948564</v>
       </c>
-      <c r="O37" t="inlineStr"/>
       <c r="P37" t="n">
         <v>6.7</v>
       </c>
@@ -2992,20 +2731,14 @@
         <v>6.65</v>
       </c>
       <c r="S37" t="n">
-        <v>6.617</v>
-      </c>
-      <c r="T37" t="inlineStr"/>
+        <v>6.305</v>
+      </c>
       <c r="U37" t="n">
         <v>5.91</v>
       </c>
       <c r="V37" t="n">
         <v>52.38</v>
       </c>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
-      <c r="Y37" t="inlineStr"/>
-      <c r="Z37" t="inlineStr"/>
-      <c r="AA37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -3021,7 +2754,7 @@
         <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>4.310000437185504</v>
+        <v>4.49</v>
       </c>
       <c r="F38" t="n">
         <v>4.37</v>
@@ -3050,7 +2783,6 @@
       <c r="N38" t="n">
         <v>1.720159303405957</v>
       </c>
-      <c r="O38" t="inlineStr"/>
       <c r="P38" t="n">
         <v>5.71</v>
       </c>
@@ -3061,20 +2793,14 @@
         <v>5.66</v>
       </c>
       <c r="S38" t="n">
-        <v>5.627</v>
-      </c>
-      <c r="T38" t="inlineStr"/>
+        <v>5.757</v>
+      </c>
       <c r="U38" t="n">
         <v>5.86</v>
       </c>
       <c r="V38" t="n">
         <v>51.94</v>
       </c>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
-      <c r="Y38" t="inlineStr"/>
-      <c r="Z38" t="inlineStr"/>
-      <c r="AA38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -3090,7 +2816,7 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>4.379999471528501</v>
+        <v>4.374</v>
       </c>
       <c r="F39" t="n">
         <v>0</v>
@@ -3098,22 +2824,18 @@
       <c r="G39" t="n">
         <v>1</v>
       </c>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="n">
         <v>0</v>
       </c>
       <c r="J39" t="n">
         <v>1</v>
       </c>
-      <c r="K39" t="inlineStr"/>
       <c r="L39" t="n">
         <v>0</v>
       </c>
       <c r="M39" t="n">
         <v>1</v>
       </c>
-      <c r="N39" t="inlineStr"/>
-      <c r="O39" t="inlineStr"/>
       <c r="P39" t="n">
         <v>5.85</v>
       </c>
@@ -3124,20 +2846,14 @@
         <v>5.8</v>
       </c>
       <c r="S39" t="n">
-        <v>5.767</v>
-      </c>
-      <c r="T39" t="inlineStr"/>
+        <v>5.773</v>
+      </c>
       <c r="U39" t="n">
         <v>5.88</v>
       </c>
       <c r="V39" t="n">
         <v>52.01</v>
       </c>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
-      <c r="Y39" t="inlineStr"/>
-      <c r="Z39" t="inlineStr"/>
-      <c r="AA39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -3153,7 +2869,7 @@
         <v>1</v>
       </c>
       <c r="E40" t="n">
-        <v>4.449999548310974</v>
+        <v>4.489</v>
       </c>
       <c r="F40" t="n">
         <v>6.03</v>
@@ -3182,7 +2898,6 @@
       <c r="N40" t="n">
         <v>1.859738566197147</v>
       </c>
-      <c r="O40" t="inlineStr"/>
       <c r="P40" t="n">
         <v>5.99</v>
       </c>
@@ -3193,20 +2908,14 @@
         <v>5.94</v>
       </c>
       <c r="S40" t="n">
-        <v>5.907</v>
-      </c>
-      <c r="T40" t="inlineStr"/>
+        <v>6.185</v>
+      </c>
       <c r="U40" t="n">
         <v>5.89</v>
       </c>
       <c r="V40" t="n">
         <v>52.08</v>
       </c>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
-      <c r="Y40" t="inlineStr"/>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -3222,7 +2931,7 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>4.519999840669676</v>
+        <v>4.588</v>
       </c>
       <c r="F41" t="n">
         <v>7.08</v>
@@ -3251,7 +2960,6 @@
       <c r="N41" t="n">
         <v>1.929929560084588</v>
       </c>
-      <c r="O41" t="inlineStr"/>
       <c r="P41" t="n">
         <v>6.13</v>
       </c>
@@ -3262,20 +2970,14 @@
         <v>6.08</v>
       </c>
       <c r="S41" t="n">
-        <v>6.047</v>
-      </c>
-      <c r="T41" t="inlineStr"/>
+        <v>5.429</v>
+      </c>
       <c r="U41" t="n">
         <v>5.91</v>
       </c>
       <c r="V41" t="n">
         <v>52.15</v>
       </c>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
-      <c r="Y41" t="inlineStr"/>
-      <c r="Z41" t="inlineStr"/>
-      <c r="AA41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -3291,7 +2993,7 @@
         <v>1</v>
       </c>
       <c r="E42" t="n">
-        <v>4.589999838141592</v>
+        <v>4.586</v>
       </c>
       <c r="F42" t="n">
         <v>8.32</v>
@@ -3320,7 +3022,6 @@
       <c r="N42" t="n">
         <v>2</v>
       </c>
-      <c r="O42" t="inlineStr"/>
       <c r="P42" t="n">
         <v>6.27</v>
       </c>
@@ -3331,20 +3032,14 @@
         <v>6.22</v>
       </c>
       <c r="S42" t="n">
-        <v>6.187</v>
-      </c>
-      <c r="T42" t="inlineStr"/>
+        <v>5.634</v>
+      </c>
       <c r="U42" t="n">
         <v>5.93</v>
       </c>
       <c r="V42" t="n">
         <v>52.22</v>
       </c>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
-      <c r="Y42" t="inlineStr"/>
-      <c r="Z42" t="inlineStr"/>
-      <c r="AA42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -3360,7 +3055,7 @@
         <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>4.609999703842231</v>
+        <v>4.779</v>
       </c>
       <c r="F43" t="n">
         <v>0</v>
@@ -3368,22 +3063,18 @@
       <c r="G43" t="n">
         <v>1</v>
       </c>
-      <c r="H43" t="inlineStr"/>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" t="n">
         <v>1</v>
       </c>
-      <c r="K43" t="inlineStr"/>
       <c r="L43" t="n">
         <v>0</v>
       </c>
       <c r="M43" t="n">
         <v>1</v>
       </c>
-      <c r="N43" t="inlineStr"/>
-      <c r="O43" t="inlineStr"/>
       <c r="P43" t="n">
         <v>5.28</v>
       </c>
@@ -3394,20 +3085,14 @@
         <v>5.23</v>
       </c>
       <c r="S43" t="n">
-        <v>5.197</v>
-      </c>
-      <c r="T43" t="inlineStr"/>
+        <v>5.676</v>
+      </c>
       <c r="U43" t="n">
         <v>5.88</v>
       </c>
       <c r="V43" t="n">
         <v>51.78</v>
       </c>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
-      <c r="Y43" t="inlineStr"/>
-      <c r="Z43" t="inlineStr"/>
-      <c r="AA43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -3423,7 +3108,7 @@
         <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>4.67999991622922</v>
+        <v>4.919</v>
       </c>
       <c r="F44" t="n">
         <v>7.94</v>
@@ -3452,7 +3137,6 @@
       <c r="N44" t="n">
         <v>1.9698816437465</v>
       </c>
-      <c r="O44" t="inlineStr"/>
       <c r="P44" t="n">
         <v>5.42</v>
       </c>
@@ -3463,20 +3147,14 @@
         <v>5.37</v>
       </c>
       <c r="S44" t="n">
-        <v>5.337</v>
-      </c>
-      <c r="T44" t="inlineStr"/>
+        <v>5.222</v>
+      </c>
       <c r="U44" t="n">
         <v>5.9</v>
       </c>
       <c r="V44" t="n">
         <v>51.85</v>
       </c>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
-      <c r="Y44" t="inlineStr"/>
-      <c r="Z44" t="inlineStr"/>
-      <c r="AA44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -3492,7 +3170,7 @@
         <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>4.749999748856418</v>
+        <v>4.673</v>
       </c>
       <c r="F45" t="n">
         <v>9.33</v>
@@ -3521,7 +3199,6 @@
       <c r="N45" t="n">
         <v>2.03981055414835</v>
       </c>
-      <c r="O45" t="inlineStr"/>
       <c r="P45" t="n">
         <v>5.56</v>
       </c>
@@ -3532,20 +3209,14 @@
         <v>5.51</v>
       </c>
       <c r="S45" t="n">
-        <v>5.477</v>
-      </c>
-      <c r="T45" t="inlineStr"/>
+        <v>5.619</v>
+      </c>
       <c r="U45" t="n">
         <v>5.92</v>
       </c>
       <c r="V45" t="n">
         <v>51.92</v>
       </c>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
-      <c r="Y45" t="inlineStr"/>
-      <c r="Z45" t="inlineStr"/>
-      <c r="AA45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -3561,7 +3232,7 @@
         <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>4.819999705510486</v>
+        <v>4.814</v>
       </c>
       <c r="F46" t="n">
         <v>10.96</v>
@@ -3590,7 +3261,6 @@
       <c r="N46" t="n">
         <v>2.109915863023793</v>
       </c>
-      <c r="O46" t="inlineStr"/>
       <c r="P46" t="n">
         <v>5.7</v>
       </c>
@@ -3601,20 +3271,14 @@
         <v>5.65</v>
       </c>
       <c r="S46" t="n">
-        <v>5.617</v>
-      </c>
-      <c r="T46" t="inlineStr"/>
+        <v>5.167</v>
+      </c>
       <c r="U46" t="n">
         <v>5.94</v>
       </c>
       <c r="V46" t="n">
         <v>51.99</v>
       </c>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
-      <c r="Y46" t="inlineStr"/>
-      <c r="Z46" t="inlineStr"/>
-      <c r="AA46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -3630,7 +3294,7 @@
         <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>4.889999934748613</v>
+        <v>4.824</v>
       </c>
       <c r="F47" t="n">
         <v>12.88</v>
@@ -3659,7 +3323,6 @@
       <c r="N47" t="n">
         <v>2.180125875164054</v>
       </c>
-      <c r="O47" t="inlineStr"/>
       <c r="P47" t="n">
         <v>5.84</v>
       </c>
@@ -3670,20 +3333,14 @@
         <v>5.79</v>
       </c>
       <c r="S47" t="n">
-        <v>5.757</v>
-      </c>
-      <c r="T47" t="inlineStr"/>
+        <v>5.375</v>
+      </c>
       <c r="U47" t="n">
         <v>5.96</v>
       </c>
       <c r="V47" t="n">
         <v>52.06</v>
       </c>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
-      <c r="Y47" t="inlineStr"/>
-      <c r="Z47" t="inlineStr"/>
-      <c r="AA47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -3699,7 +3356,7 @@
         <v>1</v>
       </c>
       <c r="E48" t="n">
-        <v>4.910000258512931</v>
+        <v>5.157</v>
       </c>
       <c r="F48" t="n">
         <v>10.47</v>
@@ -3728,7 +3385,6 @@
       <c r="N48" t="n">
         <v>2.079904467666721</v>
       </c>
-      <c r="O48" t="inlineStr"/>
       <c r="P48" t="n">
         <v>4.85</v>
       </c>
@@ -3739,20 +3395,14 @@
         <v>4.8</v>
       </c>
       <c r="S48" t="n">
-        <v>4.767</v>
-      </c>
-      <c r="T48" t="inlineStr"/>
+        <v>5.008</v>
+      </c>
       <c r="U48" t="n">
         <v>5.91</v>
       </c>
       <c r="V48" t="n">
         <v>51.62</v>
       </c>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
-      <c r="Y48" t="inlineStr"/>
-      <c r="Z48" t="inlineStr"/>
-      <c r="AA48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -3768,7 +3418,7 @@
         <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>4.980000188261741</v>
+        <v>5.074</v>
       </c>
       <c r="F49" t="n">
         <v>12.3</v>
@@ -3797,7 +3447,6 @@
       <c r="N49" t="n">
         <v>2.150142161848559</v>
       </c>
-      <c r="O49" t="inlineStr"/>
       <c r="P49" t="n">
         <v>4.99</v>
       </c>
@@ -3808,20 +3457,14 @@
         <v>4.94</v>
       </c>
       <c r="S49" t="n">
-        <v>4.907</v>
-      </c>
-      <c r="T49" t="inlineStr"/>
+        <v>4.904</v>
+      </c>
       <c r="U49" t="n">
         <v>5.93</v>
       </c>
       <c r="V49" t="n">
         <v>51.69</v>
       </c>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
-      <c r="Y49" t="inlineStr"/>
-      <c r="Z49" t="inlineStr"/>
-      <c r="AA49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -3837,7 +3480,7 @@
         <v>1</v>
       </c>
       <c r="E50" t="n">
-        <v>5.049999824155409</v>
+        <v>5.157</v>
       </c>
       <c r="F50" t="n">
         <v>14.45</v>
@@ -3866,7 +3509,6 @@
       <c r="N50" t="n">
         <v>2.220108088040055</v>
       </c>
-      <c r="O50" t="inlineStr"/>
       <c r="P50" t="n">
         <v>5.13</v>
       </c>
@@ -3877,20 +3519,14 @@
         <v>5.08</v>
       </c>
       <c r="S50" t="n">
-        <v>5.047</v>
-      </c>
-      <c r="T50" t="inlineStr"/>
+        <v>5.155</v>
+      </c>
       <c r="U50" t="n">
         <v>5.94</v>
       </c>
       <c r="V50" t="n">
         <v>51.76</v>
       </c>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
-      <c r="Y50" t="inlineStr"/>
-      <c r="Z50" t="inlineStr"/>
-      <c r="AA50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -3906,7 +3542,7 @@
         <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>5.120000086131552</v>
+        <v>5.059</v>
       </c>
       <c r="F51" t="n">
         <v>16.98</v>
@@ -3935,7 +3571,6 @@
       <c r="N51" t="n">
         <v>2.290034611362518</v>
       </c>
-      <c r="O51" t="inlineStr"/>
       <c r="P51" t="n">
         <v>5.27</v>
       </c>
@@ -3946,20 +3581,14 @@
         <v>5.22</v>
       </c>
       <c r="S51" t="n">
-        <v>5.187</v>
-      </c>
-      <c r="T51" t="inlineStr"/>
+        <v>4.805</v>
+      </c>
       <c r="U51" t="n">
         <v>5.96</v>
       </c>
       <c r="V51" t="n">
         <v>51.83</v>
       </c>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
-      <c r="Y51" t="inlineStr"/>
-      <c r="Z51" t="inlineStr"/>
-      <c r="AA51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -3975,7 +3604,7 @@
         <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>5.190000106858478</v>
+        <v>4.985</v>
       </c>
       <c r="F52" t="n">
         <v>19.95</v>
@@ -4004,7 +3633,6 @@
       <c r="N52" t="n">
         <v>2.360025089189397</v>
       </c>
-      <c r="O52" t="inlineStr"/>
       <c r="P52" t="n">
         <v>5.41</v>
       </c>
@@ -4015,20 +3643,14 @@
         <v>5.36</v>
       </c>
       <c r="S52" t="n">
-        <v>5.327</v>
-      </c>
-      <c r="T52" t="inlineStr"/>
+        <v>4.707</v>
+      </c>
       <c r="U52" t="n">
         <v>5.98</v>
       </c>
       <c r="V52" t="n">
         <v>51.9</v>
       </c>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
-      <c r="Y52" t="inlineStr"/>
-      <c r="Z52" t="inlineStr"/>
-      <c r="AA52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -4073,23 +3695,12 @@
       <c r="N53" t="n">
         <v>2.260071387985075</v>
       </c>
-      <c r="O53" t="inlineStr"/>
-      <c r="P53" t="inlineStr"/>
-      <c r="Q53" t="inlineStr"/>
-      <c r="R53" t="inlineStr"/>
-      <c r="S53" t="inlineStr"/>
-      <c r="T53" t="inlineStr"/>
       <c r="U53" t="n">
         <v>5.93</v>
       </c>
       <c r="V53" t="n">
         <v>51.46</v>
       </c>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
-      <c r="Y53" t="inlineStr"/>
-      <c r="Z53" t="inlineStr"/>
-      <c r="AA53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -4134,23 +3745,12 @@
       <c r="N54" t="n">
         <v>2.330007700872759</v>
       </c>
-      <c r="O54" t="inlineStr"/>
-      <c r="P54" t="inlineStr"/>
-      <c r="Q54" t="inlineStr"/>
-      <c r="R54" t="inlineStr"/>
-      <c r="S54" t="inlineStr"/>
-      <c r="T54" t="inlineStr"/>
       <c r="U54" t="n">
         <v>5.95</v>
       </c>
       <c r="V54" t="n">
         <v>51.53</v>
       </c>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
-      <c r="Y54" t="inlineStr"/>
-      <c r="Z54" t="inlineStr"/>
-      <c r="AA54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -4195,23 +3795,12 @@
       <c r="N55" t="n">
         <v>2.400019635065159</v>
       </c>
-      <c r="O55" t="inlineStr"/>
-      <c r="P55" t="inlineStr"/>
-      <c r="Q55" t="inlineStr"/>
-      <c r="R55" t="inlineStr"/>
-      <c r="S55" t="inlineStr"/>
-      <c r="T55" t="inlineStr"/>
       <c r="U55" t="n">
         <v>5.97</v>
       </c>
       <c r="V55" t="n">
         <v>51.6</v>
       </c>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
-      <c r="Y55" t="inlineStr"/>
-      <c r="Z55" t="inlineStr"/>
-      <c r="AA55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -4256,23 +3845,12 @@
       <c r="N56" t="n">
         <v>2.469969209499959</v>
       </c>
-      <c r="O56" t="inlineStr"/>
-      <c r="P56" t="inlineStr"/>
-      <c r="Q56" t="inlineStr"/>
-      <c r="R56" t="inlineStr"/>
-      <c r="S56" t="inlineStr"/>
-      <c r="T56" t="inlineStr"/>
       <c r="U56" t="n">
         <v>5.99</v>
       </c>
       <c r="V56" t="n">
         <v>51.67</v>
       </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
-      <c r="Y56" t="inlineStr"/>
-      <c r="Z56" t="inlineStr"/>
-      <c r="AA56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -4317,23 +3895,12 @@
       <c r="N57" t="n">
         <v>2.539953841656397</v>
       </c>
-      <c r="O57" t="inlineStr"/>
-      <c r="P57" t="inlineStr"/>
-      <c r="Q57" t="inlineStr"/>
-      <c r="R57" t="inlineStr"/>
-      <c r="S57" t="inlineStr"/>
-      <c r="T57" t="inlineStr"/>
       <c r="U57" t="n">
         <v>6</v>
       </c>
       <c r="V57" t="n">
         <v>51.74</v>
       </c>
-      <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr"/>
-      <c r="Y57" t="inlineStr"/>
-      <c r="Z57" t="inlineStr"/>
-      <c r="AA57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -4378,23 +3945,12 @@
       <c r="N58" t="n">
         <v>2.439963935920905</v>
       </c>
-      <c r="O58" t="inlineStr"/>
-      <c r="P58" t="inlineStr"/>
-      <c r="Q58" t="inlineStr"/>
-      <c r="R58" t="inlineStr"/>
-      <c r="S58" t="inlineStr"/>
-      <c r="T58" t="inlineStr"/>
       <c r="U58" t="n">
         <v>5.96</v>
       </c>
       <c r="V58" t="n">
         <v>51.3</v>
       </c>
-      <c r="W58" t="inlineStr"/>
-      <c r="X58" t="inlineStr"/>
-      <c r="Y58" t="inlineStr"/>
-      <c r="Z58" t="inlineStr"/>
-      <c r="AA58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -4439,23 +3995,12 @@
       <c r="N59" t="n">
         <v>2.510008512940235</v>
       </c>
-      <c r="O59" t="inlineStr"/>
-      <c r="P59" t="inlineStr"/>
-      <c r="Q59" t="inlineStr"/>
-      <c r="R59" t="inlineStr"/>
-      <c r="S59" t="inlineStr"/>
-      <c r="T59" t="inlineStr"/>
       <c r="U59" t="n">
         <v>5.98</v>
       </c>
       <c r="V59" t="n">
         <v>51.37</v>
       </c>
-      <c r="W59" t="inlineStr"/>
-      <c r="X59" t="inlineStr"/>
-      <c r="Y59" t="inlineStr"/>
-      <c r="Z59" t="inlineStr"/>
-      <c r="AA59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -4500,23 +4045,12 @@
       <c r="N60" t="n">
         <v>2.580012112529424</v>
       </c>
-      <c r="O60" t="inlineStr"/>
-      <c r="P60" t="inlineStr"/>
-      <c r="Q60" t="inlineStr"/>
-      <c r="R60" t="inlineStr"/>
-      <c r="S60" t="inlineStr"/>
-      <c r="T60" t="inlineStr"/>
       <c r="U60" t="n">
         <v>6</v>
       </c>
       <c r="V60" t="n">
         <v>51.44</v>
       </c>
-      <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr"/>
-      <c r="Y60" t="inlineStr"/>
-      <c r="Z60" t="inlineStr"/>
-      <c r="AA60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -4561,23 +4095,12 @@
       <c r="N61" t="n">
         <v>2.650015952471839</v>
       </c>
-      <c r="O61" t="inlineStr"/>
-      <c r="P61" t="inlineStr"/>
-      <c r="Q61" t="inlineStr"/>
-      <c r="R61" t="inlineStr"/>
-      <c r="S61" t="inlineStr"/>
-      <c r="T61" t="inlineStr"/>
       <c r="U61" t="n">
         <v>6.01</v>
       </c>
       <c r="V61" t="n">
         <v>51.51</v>
       </c>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr"/>
-      <c r="Y61" t="inlineStr"/>
-      <c r="Z61" t="inlineStr"/>
-      <c r="AA61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -4622,23 +4145,12 @@
       <c r="N62" t="n">
         <v>2.719993826367604</v>
       </c>
-      <c r="O62" t="inlineStr"/>
-      <c r="P62" t="inlineStr"/>
-      <c r="Q62" t="inlineStr"/>
-      <c r="R62" t="inlineStr"/>
-      <c r="S62" t="inlineStr"/>
-      <c r="T62" t="inlineStr"/>
       <c r="U62" t="n">
         <v>6.03</v>
       </c>
       <c r="V62" t="n">
         <v>51.58</v>
       </c>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
-      <c r="Y62" t="inlineStr"/>
-      <c r="Z62" t="inlineStr"/>
-      <c r="AA62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -4683,23 +4195,12 @@
       <c r="N63" t="n">
         <v>2.620031895126298</v>
       </c>
-      <c r="O63" t="inlineStr"/>
-      <c r="P63" t="inlineStr"/>
-      <c r="Q63" t="inlineStr"/>
-      <c r="R63" t="inlineStr"/>
-      <c r="S63" t="inlineStr"/>
-      <c r="T63" t="inlineStr"/>
       <c r="U63" t="n">
         <v>5.98</v>
       </c>
       <c r="V63" t="n">
         <v>51.14</v>
       </c>
-      <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr"/>
-      <c r="Y63" t="inlineStr"/>
-      <c r="Z63" t="inlineStr"/>
-      <c r="AA63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -4744,23 +4245,12 @@
       <c r="N64" t="n">
         <v>2.690018780788695</v>
       </c>
-      <c r="O64" t="inlineStr"/>
-      <c r="P64" t="inlineStr"/>
-      <c r="Q64" t="inlineStr"/>
-      <c r="R64" t="inlineStr"/>
-      <c r="S64" t="inlineStr"/>
-      <c r="T64" t="inlineStr"/>
       <c r="U64" t="n">
         <v>6</v>
       </c>
       <c r="V64" t="n">
         <v>51.21</v>
       </c>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
-      <c r="Y64" t="inlineStr"/>
-      <c r="Z64" t="inlineStr"/>
-      <c r="AA64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -4805,23 +4295,12 @@
       <c r="N65" t="n">
         <v>2.759969857554307</v>
       </c>
-      <c r="O65" t="inlineStr"/>
-      <c r="P65" t="inlineStr"/>
-      <c r="Q65" t="inlineStr"/>
-      <c r="R65" t="inlineStr"/>
-      <c r="S65" t="inlineStr"/>
-      <c r="T65" t="inlineStr"/>
       <c r="U65" t="n">
         <v>6.02</v>
       </c>
       <c r="V65" t="n">
         <v>51.28</v>
       </c>
-      <c r="W65" t="inlineStr"/>
-      <c r="X65" t="inlineStr"/>
-      <c r="Y65" t="inlineStr"/>
-      <c r="Z65" t="inlineStr"/>
-      <c r="AA65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -4866,23 +4345,12 @@
       <c r="N66" t="n">
         <v>2.830010935936118</v>
       </c>
-      <c r="O66" t="inlineStr"/>
-      <c r="P66" t="inlineStr"/>
-      <c r="Q66" t="inlineStr"/>
-      <c r="R66" t="inlineStr"/>
-      <c r="S66" t="inlineStr"/>
-      <c r="T66" t="inlineStr"/>
       <c r="U66" t="n">
         <v>6.04</v>
       </c>
       <c r="V66" t="n">
         <v>51.35</v>
       </c>
-      <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
-      <c r="Y66" t="inlineStr"/>
-      <c r="Z66" t="inlineStr"/>
-      <c r="AA66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -4927,23 +4395,12 @@
       <c r="N67" t="n">
         <v>2.899984562549391</v>
       </c>
-      <c r="O67" t="inlineStr"/>
-      <c r="P67" t="inlineStr"/>
-      <c r="Q67" t="inlineStr"/>
-      <c r="R67" t="inlineStr"/>
-      <c r="S67" t="inlineStr"/>
-      <c r="T67" t="inlineStr"/>
       <c r="U67" t="n">
         <v>6.05</v>
       </c>
       <c r="V67" t="n">
         <v>51.42</v>
       </c>
-      <c r="W67" t="inlineStr"/>
-      <c r="X67" t="inlineStr"/>
-      <c r="Y67" t="inlineStr"/>
-      <c r="Z67" t="inlineStr"/>
-      <c r="AA67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -4988,23 +4445,12 @@
       <c r="N68" t="n">
         <v>2.800029359244134</v>
       </c>
-      <c r="O68" t="inlineStr"/>
-      <c r="P68" t="inlineStr"/>
-      <c r="Q68" t="inlineStr"/>
-      <c r="R68" t="inlineStr"/>
-      <c r="S68" t="inlineStr"/>
-      <c r="T68" t="inlineStr"/>
       <c r="U68" t="n">
         <v>6.01</v>
       </c>
       <c r="V68" t="n">
         <v>50.98</v>
       </c>
-      <c r="W68" t="inlineStr"/>
-      <c r="X68" t="inlineStr"/>
-      <c r="Y68" t="inlineStr"/>
-      <c r="Z68" t="inlineStr"/>
-      <c r="AA68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -5049,23 +4495,12 @@
       <c r="N69" t="n">
         <v>2.869994000121742</v>
       </c>
-      <c r="O69" t="inlineStr"/>
-      <c r="P69" t="inlineStr"/>
-      <c r="Q69" t="inlineStr"/>
-      <c r="R69" t="inlineStr"/>
-      <c r="S69" t="inlineStr"/>
-      <c r="T69" t="inlineStr"/>
       <c r="U69" t="n">
         <v>6.03</v>
       </c>
       <c r="V69" t="n">
         <v>51.05</v>
       </c>
-      <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
-      <c r="Y69" t="inlineStr"/>
-      <c r="Z69" t="inlineStr"/>
-      <c r="AA69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -5110,23 +4545,12 @@
       <c r="N70" t="n">
         <v>2.940018155007663</v>
       </c>
-      <c r="O70" t="inlineStr"/>
-      <c r="P70" t="inlineStr"/>
-      <c r="Q70" t="inlineStr"/>
-      <c r="R70" t="inlineStr"/>
-      <c r="S70" t="inlineStr"/>
-      <c r="T70" t="inlineStr"/>
       <c r="U70" t="n">
         <v>6.04</v>
       </c>
       <c r="V70" t="n">
         <v>51.12</v>
       </c>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
-      <c r="Y70" t="inlineStr"/>
-      <c r="Z70" t="inlineStr"/>
-      <c r="AA70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -5171,23 +4595,12 @@
       <c r="N71" t="n">
         <v>3.01000297412706</v>
       </c>
-      <c r="O71" t="inlineStr"/>
-      <c r="P71" t="inlineStr"/>
-      <c r="Q71" t="inlineStr"/>
-      <c r="R71" t="inlineStr"/>
-      <c r="S71" t="inlineStr"/>
-      <c r="T71" t="inlineStr"/>
       <c r="U71" t="n">
         <v>6.06</v>
       </c>
       <c r="V71" t="n">
         <v>51.19</v>
       </c>
-      <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
-      <c r="Y71" t="inlineStr"/>
-      <c r="Z71" t="inlineStr"/>
-      <c r="AA71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -5211,38 +4624,24 @@
       <c r="G72" t="n">
         <v>1</v>
       </c>
-      <c r="H72" t="inlineStr"/>
       <c r="I72" t="n">
         <v>0</v>
       </c>
       <c r="J72" t="n">
         <v>1</v>
       </c>
-      <c r="K72" t="inlineStr"/>
       <c r="L72" t="n">
         <v>0</v>
       </c>
       <c r="M72" t="n">
         <v>1</v>
       </c>
-      <c r="N72" t="inlineStr"/>
-      <c r="O72" t="inlineStr"/>
-      <c r="P72" t="inlineStr"/>
-      <c r="Q72" t="inlineStr"/>
-      <c r="R72" t="inlineStr"/>
-      <c r="S72" t="inlineStr"/>
-      <c r="T72" t="inlineStr"/>
       <c r="U72" t="n">
         <v>6.08</v>
       </c>
       <c r="V72" t="n">
         <v>51.26</v>
       </c>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
-      <c r="Y72" t="inlineStr"/>
-      <c r="Z72" t="inlineStr"/>
-      <c r="AA72" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>